<commit_message>
Contenidos_Consultados: PREFIJOS_AGRUPAR vacio + RULENAMES_PRESERVAR (Turnos SAP / Mis profesionales)
</commit_message>
<xml_diff>
--- a/Contenidos_Consultados/output/contenidos_consultados_abril_2026.xlsx
+++ b/Contenidos_Consultados/output/contenidos_consultados_abril_2026.xlsx
@@ -585,13 +585,13 @@
           <t>1- Confirmación Turnos Salud: (400.199)
 2- Infracciones: (190.466)
 3- Turnos Salud: (171.480)
-4- Trámites Vehículos SAP: (119.401)
-5- Hospitales: (78.347)
-6- Trámites SAP: (71.942)
-7- Licencias: (69.182)
-8- Mis profesionales: (64.955)
-9- Vacunación: (48.834)
-10- Buscar donde está permitido estacionar: (48.580)</t>
+4- Turnos SAP: (121.794)
+5- Trámites Vehículos SAP: (119.401)
+6- Mis profesionales: (106.667)
+7- Hospitales: (78.347)
+8- Trámites SAP: (71.942)
+9- Licencias: (69.182)
+10- Vacunación: (48.834)</t>
         </is>
       </c>
     </row>

</xml_diff>